<commit_message>
:card_file_box: Unity 버전 6000.2.6f2로 마이그레이션
</commit_message>
<xml_diff>
--- a/Assets/Resources/GameData/BarGuestDB.xlsx
+++ b/Assets/Resources/GameData/BarGuestDB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\UnityMyGame\Nemesis1842\Assets\Resources\GameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3A5E94-B9F7-4708-9844-87F0986FD908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA29CCB-E252-47EA-A408-7BACF1024F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="650" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guests" sheetId="2" r:id="rId1"/>

</xml_diff>